<commit_message>
Hook fleet per-registration block + J Fisher/NMS age-band x category breakdown (PF 16/07); fix duplicate 19th day label
- queries.py: hook_fleet/hook_split (area=HOOKS, reconciles with cover HOOKS row),
  fisher_nms_split (band x parts category, MTD + today, Unregistered/Plant for no-VRM lines)
- build_report.py: cover hook block rows 81+, two breakdown tabs, PDF pages 4-6
  (Fisher, NMS, Hook Fleet), day-by-day moves to page 7
- blank_template.xlsx: row 2 day labels corrected (18th was duplicated as 19th)

Tested end-to-end against July MTD data; 17 July rebuild matches production send (£6,380.33, balanced).
</commit_message>
<xml_diff>
--- a/blank_template.xlsx
+++ b/blank_template.xlsx
@@ -1,30 +1,30 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="707" firstSheet="7" activeTab="18" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Cover" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Fox Wagons" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Leyland Wagons" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="JA Jackson" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="JJ O'Grady Civils" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="J FISHER" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="J Fisher Plant" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="NMS CIVIL" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="NMS Plant" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Plant" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Graphics" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="PPE- Workwear" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Tyres" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Misc" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Damage" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Windscreen &amp; Glass" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="Assets For sale" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="Asphalt Plant " sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="Capital" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fox Wagons" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leyland Wagons" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="JA Jackson" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="JJ O'Grady Civils" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="J FISHER" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="J Fisher Plant" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NMS CIVIL" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NMS Plant" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plant" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Graphics" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PPE- Workwear" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tyres" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Misc" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Damage" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Windscreen &amp; Glass" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets For sale" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Asphalt Plant " sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capital" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1" forceFullCalc="1"/>
@@ -622,7 +622,7 @@
       </c>
       <c r="S2" s="1" t="inlineStr">
         <is>
-          <t>19th</t>
+          <t>18th</t>
         </is>
       </c>
       <c r="T2" s="1" t="inlineStr">

</xml_diff>

<commit_message>
Reference-missing overhaul + averages page + email averages
- Rename UNIDENTIFIED area to REFERENCE MISSING everywhere (cover, PDF, email,
  line review). Honest, actionable label for lines with no usable PO reference.
- get_area: apply agreed ownership rules (any 'martin' -> Plant, swarf/hitachi/
  carrington/wirtgen -> Plant, Gemini -> Workshop, trailer numbers -> Trailers,
  tyres, oil pump-ins -> Consumables) routing to existing cover rows so the
  cover still balances. Genuine unknowns stay REFERENCE MISSING, not a catch-all.
- Add CONSUMABLES as its own cover-area row (row 69; total moved to 70).
- PDF: move Average Spend per Day to page 2 with per-age and per-area bar charts.
- Email body: age-range and area averages, omitting anything under 100/day.
- Spreadsheet Trends tab: charts laid out in a 2x2 grid, no overlap.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/blank_template.xlsx
+++ b/blank_template.xlsx
@@ -504,7 +504,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AU69"/>
+  <dimension ref="A1:AU70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="37" customWidth="1" min="1" max="1"/>
@@ -4477,7 +4477,7 @@
     <row r="57" customFormat="1" s="2">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>UNIDENTIFIED</t>
+          <t>REFERENCE MISSING</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -5723,139 +5723,152 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" t="inlineStr">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>CONSUMABLES</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>0</v>
+      </c>
+      <c r="C69" t="n">
+        <v>0</v>
+      </c>
+      <c r="D69" t="n">
+        <v>0</v>
+      </c>
+      <c r="E69" t="n">
+        <v>0</v>
+      </c>
+      <c r="F69" t="n">
+        <v>0</v>
+      </c>
+      <c r="G69" t="n">
+        <v>0</v>
+      </c>
+      <c r="H69" t="n">
+        <v>0</v>
+      </c>
+      <c r="I69" t="n">
+        <v>0</v>
+      </c>
+      <c r="J69" t="n">
+        <v>0</v>
+      </c>
+      <c r="K69" t="n">
+        <v>0</v>
+      </c>
+      <c r="L69" t="n">
+        <v>0</v>
+      </c>
+      <c r="M69" t="n">
+        <v>0</v>
+      </c>
+      <c r="N69" t="n">
+        <v>0</v>
+      </c>
+      <c r="O69" t="n">
+        <v>0</v>
+      </c>
+      <c r="P69" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q69" t="n">
+        <v>0</v>
+      </c>
+      <c r="R69" t="n">
+        <v>0</v>
+      </c>
+      <c r="S69" t="n">
+        <v>0</v>
+      </c>
+      <c r="T69" t="n">
+        <v>0</v>
+      </c>
+      <c r="U69" t="n">
+        <v>0</v>
+      </c>
+      <c r="V69" t="n">
+        <v>0</v>
+      </c>
+      <c r="W69" t="n">
+        <v>0</v>
+      </c>
+      <c r="X69" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y69" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI69" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
         <is>
           <t>Area Total</t>
         </is>
       </c>
-      <c r="B69" s="2">
-        <f>SUM(B47:B68)</f>
-        <v/>
-      </c>
-      <c r="C69" s="2">
-        <f>SUM(C47:C68)</f>
-        <v/>
-      </c>
-      <c r="D69" s="2">
-        <f>SUM(D47:D68)</f>
-        <v/>
-      </c>
-      <c r="E69" s="2">
-        <f>SUM(E47:E68)</f>
-        <v/>
-      </c>
-      <c r="F69" s="2">
-        <f>SUM(F47:F68)</f>
-        <v/>
-      </c>
-      <c r="G69" s="2">
-        <f>SUM(G47:G68)</f>
-        <v/>
-      </c>
-      <c r="H69" s="2">
-        <f>SUM(H47:H68)</f>
-        <v/>
-      </c>
-      <c r="I69" s="2">
-        <f>SUM(I47:I68)</f>
-        <v/>
-      </c>
-      <c r="J69" s="2">
-        <f>SUM(J47:J68)</f>
-        <v/>
-      </c>
-      <c r="K69" s="2">
-        <f>SUM(K47:K68)</f>
-        <v/>
-      </c>
-      <c r="L69" s="2">
-        <f>SUM(L47:L68)</f>
-        <v/>
-      </c>
-      <c r="M69" s="2">
-        <f>SUM(M47:M68)</f>
-        <v/>
-      </c>
-      <c r="N69" s="2">
-        <f>SUM(N47:N68)</f>
-        <v/>
-      </c>
-      <c r="O69" s="2">
-        <f>SUM(O47:O68)</f>
-        <v/>
-      </c>
-      <c r="P69" s="2">
-        <f>SUM(P47:P68)</f>
-        <v/>
-      </c>
-      <c r="Q69" s="2">
-        <f>SUM(Q47:Q68)</f>
-        <v/>
-      </c>
-      <c r="R69" s="2">
-        <f>SUM(R47:R68)</f>
-        <v/>
-      </c>
-      <c r="S69" s="2">
-        <f>SUM(S47:S68)</f>
-        <v/>
-      </c>
-      <c r="T69" s="2">
-        <f>SUM(T47:T68)</f>
-        <v/>
-      </c>
-      <c r="U69" s="2">
-        <f>SUM(U47:U68)</f>
-        <v/>
-      </c>
-      <c r="V69" s="2">
-        <f>SUM(V47:V68)</f>
-        <v/>
-      </c>
-      <c r="W69" s="2">
-        <f>SUM(W47:W68)</f>
-        <v/>
-      </c>
-      <c r="X69" s="2">
-        <f>SUM(X47:X68)</f>
-        <v/>
-      </c>
-      <c r="Y69" s="2">
-        <f>SUM(Y47:Y68)</f>
-        <v/>
-      </c>
-      <c r="Z69" s="2">
-        <f>SUM(Z47:Z68)</f>
-        <v/>
-      </c>
-      <c r="AA69" s="2">
-        <f>SUM(AA47:AA68)</f>
-        <v/>
-      </c>
-      <c r="AB69" s="2">
-        <f>SUM(AB47:AB68)</f>
-        <v/>
-      </c>
-      <c r="AC69" s="2">
-        <f>SUM(AC47:AC68)</f>
-        <v/>
-      </c>
-      <c r="AD69" s="2">
-        <f>SUM(AD47:AD68)</f>
-        <v/>
-      </c>
-      <c r="AE69" s="2">
-        <f>SUM(AE47:AE68)</f>
-        <v/>
-      </c>
-      <c r="AF69" s="2">
-        <f>SUM(AF47:AF68)</f>
-        <v/>
-      </c>
-      <c r="AG69" s="2">
-        <f>SUM(AG47:AG68)</f>
-        <v/>
-      </c>
+      <c r="B70" s="2" t="n"/>
+      <c r="C70" s="2" t="n"/>
+      <c r="D70" s="2" t="n"/>
+      <c r="E70" s="2" t="n"/>
+      <c r="F70" s="2" t="n"/>
+      <c r="G70" s="2" t="n"/>
+      <c r="H70" s="2" t="n"/>
+      <c r="I70" s="2" t="n"/>
+      <c r="J70" s="2" t="n"/>
+      <c r="K70" s="2" t="n"/>
+      <c r="L70" s="2" t="n"/>
+      <c r="M70" s="2" t="n"/>
+      <c r="N70" s="2" t="n"/>
+      <c r="O70" s="2" t="n"/>
+      <c r="P70" s="2" t="n"/>
+      <c r="Q70" s="2" t="n"/>
+      <c r="R70" s="2" t="n"/>
+      <c r="S70" s="2" t="n"/>
+      <c r="T70" s="2" t="n"/>
+      <c r="U70" s="2" t="n"/>
+      <c r="V70" s="2" t="n"/>
+      <c r="W70" s="2" t="n"/>
+      <c r="X70" s="2" t="n"/>
+      <c r="Y70" s="2" t="n"/>
+      <c r="Z70" s="2" t="n"/>
+      <c r="AA70" s="2" t="n"/>
+      <c r="AB70" s="2" t="n"/>
+      <c r="AC70" s="2" t="n"/>
+      <c r="AD70" s="2" t="n"/>
+      <c r="AE70" s="2" t="n"/>
+      <c r="AF70" s="2" t="n"/>
+      <c r="AG70" s="2" t="n"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="AK1:AK1048576">

</xml_diff>